<commit_message>
XD line delay 추가
</commit_message>
<xml_diff>
--- a/X-Series/XD04P/LED_Module_Control_BD/XD04_LED_Module_Control_BD/Docs/xdic_led_module_반출내역.xlsx
+++ b/X-Series/XD04P/LED_Module_Control_BD/XD04_LED_Module_Control_BD/Docs/xdic_led_module_반출내역.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XD04P\LED_Module_Control_BD\XD04_LED_Module_Control_BD\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{899357AB-148B-46A6-B9E7-EA7E4D1D4099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F917843A-4FA6-4FFD-8E2D-030A6B8487BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4213BFC1-987B-470C-A934-0A5A250397E7}"/>
+    <workbookView xWindow="43080" yWindow="2160" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4213BFC1-987B-470C-A934-0A5A250397E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
   <si>
     <t>루멘스</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -165,6 +165,18 @@
   </si>
   <si>
     <t>주페이 방문 당시 다운로드 해줬던 버전, 12/19와 차이 없음</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"26. 03. 10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>xdic_led_module_control_bd_release_260310.hex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Duty 제어 기능 추가</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -799,7 +811,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB5E52BB-E1D5-4646-A95E-7F5D1E996CD9}">
-  <dimension ref="B2:E8"/>
+  <dimension ref="B2:E9"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.58203125" customWidth="1"/>
@@ -904,6 +916,20 @@
         <v>32</v>
       </c>
     </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B9" s="4">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>